<commit_message>
Show chart axes in the report and add a screenshot to the README
openpyxl 3.1 omits the axis delete flag, so Excel hid the month names and amounts on the Summary chart. The end-to-end test now checks that both axes are visible. The example report is rebuilt with its title, and examples/summary.png shows its Summary sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/sales_report.xlsx
+++ b/examples/sales_report.xlsx
@@ -194,6 +194,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -235,6 +236,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -246,6 +248,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -262,6 +265,7 @@
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
@@ -611,7 +615,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Period 01.07.2026 to 30.09.2026. Built from 3 files on 11.10.2026 13:35.</t>
+          <t>Period 01.07.2026 to 30.09.2026. Built from 3 files on 21.10.2026 22:02.</t>
         </is>
       </c>
     </row>

</xml_diff>